<commit_message>
fixed rationalisation + unknown subfunctions handled + chatbot fixes
</commit_message>
<xml_diff>
--- a/CENSUS_RATIONALISATION/app_2/app_2/excel data/Sample output for first 50 rows.xlsx
+++ b/CENSUS_RATIONALISATION/app_2/app_2/excel data/Sample output for first 50 rows.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sshaju\Downloads\Census Data Rationalization\Requirements for DTS team\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://itinfoalvarezandmarsalind-my.sharepoint.com/personal/jagritjain_alvarezandmarsal_com/Documents/Documents/APPS/ORG_ANALYSIS/CENSUS_RATIONALISATION/app_2/app_2/excel data/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{641EE160-DD71-4E89-A8C0-44A8863BD17F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{29D02840-A618-4398-B4D5-C1D04202E550}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{29D02840-A618-4398-B4D5-C1D04202E550}"/>
   </bookViews>
   <sheets>
     <sheet name="Census_Cleansed_sample output" sheetId="1" r:id="rId1"/>
@@ -3086,15 +3086,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="c025f7fb-0507-4c58-9d21-70c81cc719d8" xsi:nil="true"/>
@@ -3103,6 +3094,15 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3341,20 +3341,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DA97CF0-1D84-427A-BCCD-B33B3A21A957}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C29367D3-6D07-4F98-A880-CCB47BC72E21}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="c025f7fb-0507-4c58-9d21-70c81cc719d8"/>
     <ds:schemaRef ds:uri="525b86ac-cf74-4994-a84b-4d7e6c8645fa"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DA97CF0-1D84-427A-BCCD-B33B3A21A957}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>